<commit_message>
update bill and where text
</commit_message>
<xml_diff>
--- a/bill/record.xlsx
+++ b/bill/record.xlsx
@@ -5,15 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhangzhm\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alantop_dir\alantop_data\alantop_git\github\bill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EEDC52-D780-4E2F-B625-FA5FAF407F30}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0DB9F28-C3E2-4CED-BE2B-D5F7F0A8330F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="10.4" sheetId="4" r:id="rId1"/>
+    <sheet name="10.3" sheetId="3" r:id="rId2"/>
+    <sheet name="10.2" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="39">
   <si>
     <t>ju</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -71,10 +73,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>悦动圈天天</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>淘宝1000红包</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -104,6 +102,86 @@
   </si>
   <si>
     <t>居支付宝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>悦动圈天天10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>悦动圈健走闯关塞10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>金额</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>序列号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>步数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>名称</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>天天走路领红包</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>刷卡银行</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>交通4057</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>好友PK赛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中信6530</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>钉钉</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>交通7493</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中信2382</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>提现否 （1提现，0未提现）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否提现</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开始摇时间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>提交健走闯关赛退出，退出时间 10.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>报名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>居中信</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -135,7 +213,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -158,17 +236,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -451,29 +586,691 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9A0F91A-D02D-457B-B3D9-48656CF541FC}">
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="11"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="13"/>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="13"/>
+      <c r="B5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
+      <c r="B8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="13"/>
+      <c r="B9" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="13"/>
+      <c r="B11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="3">
+        <v>2</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="13"/>
+      <c r="B13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D14" s="3">
+        <v>2</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="13"/>
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="9"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="12"/>
+      <c r="C21" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42BB32C-5522-47CB-89EC-BA29E49614E8}">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="5" max="5" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="I2" s="8">
+        <v>0.3034722222222222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="13"/>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3">
+        <v>3</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="13"/>
+      <c r="B5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>4</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3">
+        <v>5</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
+      <c r="B8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3">
+        <v>2</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="13"/>
+      <c r="B9" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3">
+        <v>3</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>4</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="13"/>
+      <c r="B11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3">
+        <v>5</v>
+      </c>
+      <c r="G11" s="5"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="3">
+        <v>2</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3">
+        <v>6</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="13"/>
+      <c r="B13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3">
+        <v>7</v>
+      </c>
+      <c r="G13" s="5"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D14" s="3">
+        <v>2</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3">
+        <v>8</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="13"/>
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3">
+        <v>9</v>
+      </c>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="12"/>
+      <c r="C21" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3"/>
+      <c r="C1" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>18</v>
+      <c r="E1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>1</v>
@@ -488,8 +1285,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="13"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -497,15 +1294,15 @@
         <v>10</v>
       </c>
       <c r="D3" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>19</v>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -520,8 +1317,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="13"/>
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -535,8 +1332,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -548,32 +1345,36 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>14</v>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
       <c r="E7" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3">
+        <v>1</v>
+      </c>
       <c r="E8" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="13"/>
       <c r="B9" s="3" t="s">
         <v>2</v>
       </c>
@@ -585,21 +1386,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>15</v>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
       <c r="E10" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="13"/>
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
@@ -611,47 +1414,57 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>16</v>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="C12" s="3">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
       <c r="E12" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="13"/>
       <c r="B13" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="C13" s="3">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
       <c r="E13" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>17</v>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>16</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3">
+        <v>1</v>
+      </c>
       <c r="E14" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="13"/>
       <c r="B15" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3">
@@ -663,10 +1476,10 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="1"/>
+      <c r="B20" s="12"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="1"/>
+      <c r="B21" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
update bill and soft sublime update url and install
</commit_message>
<xml_diff>
--- a/bill/record.xlsx
+++ b/bill/record.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alantop_dir\alantop_data\alantop_git\github\bill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46F15F9-DD75-4310-AD4E-F69298699611}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAE9D83-6CE4-49AC-A8A3-74E314DAB54C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="10.5 报名 Apply " sheetId="5" r:id="rId1"/>
-    <sheet name="10.4 报名 Apply" sheetId="4" r:id="rId2"/>
-    <sheet name="10.3" sheetId="3" r:id="rId3"/>
-    <sheet name="10.2" sheetId="1" r:id="rId4"/>
+    <sheet name="10.6 报名 Apply-10.7号打卡 " sheetId="7" r:id="rId1"/>
+    <sheet name="10.5 报名 Apply-10.6号打卡" sheetId="6" r:id="rId2"/>
+    <sheet name="10.4 报名 Apply " sheetId="5" r:id="rId3"/>
+    <sheet name="10.4 报名 Apply" sheetId="4" r:id="rId4"/>
+    <sheet name="10.3" sheetId="3" r:id="rId5"/>
+    <sheet name="10.2" sheetId="1" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="60">
   <si>
     <t>ju</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -215,6 +217,58 @@
   </si>
   <si>
     <t>健走闯关塞 10.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>团队印花赛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.5-10.12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.5-10.11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.5-10.6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开始时间-结束时间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>早起打卡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>平安9221 可以刷了三笔 188</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>红色为报名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.5-10.12 10.19-10.26</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.23 交通银行 超级</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.8-10.9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>居平安</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.5-10.11，10-7-10.13</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -222,7 +276,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,6 +291,13 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -246,7 +307,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -313,11 +374,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -340,7 +414,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -622,6 +712,825 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9B029A4-88A2-46C8-B0E9-E61E955E93AB}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="16"/>
+      <c r="B3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="16"/>
+      <c r="B4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D4" s="3">
+        <v>300</v>
+      </c>
+      <c r="E4" s="14">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="14">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="16"/>
+      <c r="B6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="16"/>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="18"/>
+      <c r="B10" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="14">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="19"/>
+      <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="16"/>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="18"/>
+      <c r="B15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="3">
+        <v>6666</v>
+      </c>
+      <c r="D15" s="3">
+        <v>300</v>
+      </c>
+      <c r="E15" s="14">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
+      <c r="B16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D16" s="3">
+        <v>300</v>
+      </c>
+      <c r="E16" s="14">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="19"/>
+      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A17"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1C76AF-BB5D-4CD7-A338-58E8ADB40F19}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="16"/>
+      <c r="B3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="16"/>
+      <c r="B4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D4" s="3">
+        <v>900</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="14">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="16"/>
+      <c r="B6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="16"/>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="18"/>
+      <c r="B10" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="14">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="19"/>
+      <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="16"/>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="18"/>
+      <c r="B15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="3">
+        <v>6666</v>
+      </c>
+      <c r="D15" s="3">
+        <v>300</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
+      <c r="B16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D16" s="3">
+        <v>900</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="19"/>
+      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1</v>
+      </c>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A12:A13"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC38130-5053-47EB-A0EE-B1F3AFE32D40}">
   <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
@@ -668,7 +1577,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -687,7 +1596,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
+      <c r="A3" s="16"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -704,7 +1613,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="14"/>
+      <c r="A4" s="16"/>
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -717,7 +1626,9 @@
       <c r="E4" s="3">
         <v>1</v>
       </c>
-      <c r="F4" s="3"/>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
       <c r="G4" s="3" t="s">
         <v>40</v>
       </c>
@@ -731,7 +1642,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -744,7 +1655,9 @@
       <c r="E5" s="3">
         <v>1</v>
       </c>
-      <c r="F5" s="3"/>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
       <c r="G5" s="3" t="s">
         <v>38</v>
       </c>
@@ -756,7 +1669,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="16"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -773,7 +1686,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="14"/>
+      <c r="A7" s="16"/>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
@@ -790,7 +1703,7 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -809,7 +1722,7 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
@@ -826,7 +1739,7 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="16"/>
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
@@ -837,7 +1750,9 @@
       <c r="E10" s="3">
         <v>1</v>
       </c>
-      <c r="F10" s="3"/>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
       <c r="G10" s="3" t="s">
         <v>29</v>
       </c>
@@ -849,7 +1764,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -868,7 +1783,7 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
@@ -885,7 +1800,7 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -906,7 +1821,7 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
+      <c r="A14" s="16"/>
       <c r="B14" s="3" t="s">
         <v>41</v>
       </c>
@@ -919,7 +1834,9 @@
       <c r="E14" s="3">
         <v>1</v>
       </c>
-      <c r="F14" s="3"/>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
       <c r="G14" s="3" t="s">
         <v>40</v>
       </c>
@@ -931,7 +1848,7 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="3" t="s">
         <v>39</v>
       </c>
@@ -944,7 +1861,9 @@
       <c r="E15" s="3">
         <v>1</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
       <c r="G15" s="3" t="s">
         <v>40</v>
       </c>
@@ -958,7 +1877,7 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -977,7 +1896,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
+      <c r="A17" s="16"/>
       <c r="B17" s="3" t="s">
         <v>12</v>
       </c>
@@ -995,11 +1914,11 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="13"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="12"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="13"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="12"/>
     </row>
   </sheetData>
@@ -1018,7 +1937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9A0F91A-D02D-457B-B3D9-48656CF541FC}">
   <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
@@ -1065,7 +1984,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1084,7 +2003,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
+      <c r="A3" s="16"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -1101,7 +2020,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="14"/>
+      <c r="A4" s="16"/>
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -1130,7 +2049,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -1157,7 +2076,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="16"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1174,7 +2093,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="14"/>
+      <c r="A7" s="16"/>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1191,7 +2110,7 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1210,7 +2129,7 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
@@ -1227,7 +2146,7 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="16"/>
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1252,7 +2171,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1271,7 +2190,7 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
@@ -1288,7 +2207,7 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1309,7 +2228,7 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
+      <c r="A14" s="16"/>
       <c r="B14" s="3" t="s">
         <v>45</v>
       </c>
@@ -1336,7 +2255,7 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="3" t="s">
         <v>46</v>
       </c>
@@ -1365,7 +2284,7 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1384,7 +2303,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
+      <c r="A17" s="16"/>
       <c r="B17" s="3" t="s">
         <v>12</v>
       </c>
@@ -1408,11 +2327,11 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="13"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="9"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="13"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="9"/>
     </row>
   </sheetData>
@@ -1431,7 +2350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42BB32C-5522-47CB-89EC-BA29E49614E8}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
@@ -1471,7 +2390,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1489,7 +2408,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
+      <c r="A3" s="16"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1502,7 +2421,7 @@
       <c r="G3" s="5"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -1523,7 +2442,7 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="14"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1544,7 +2463,7 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="16"/>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1565,7 +2484,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -1588,7 +2507,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="3" t="s">
         <v>28</v>
       </c>
@@ -1609,7 +2528,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="3" t="s">
         <v>2</v>
       </c>
@@ -1628,7 +2547,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -1651,7 +2570,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
@@ -1664,7 +2583,7 @@
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -1687,7 +2606,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="3" t="s">
         <v>20</v>
       </c>
@@ -1702,7 +2621,7 @@
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1725,7 +2644,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -1747,11 +2666,11 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="13"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="1"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="13"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="1"/>
     </row>
   </sheetData>
@@ -1770,7 +2689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
@@ -1800,7 +2719,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1817,7 +2736,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
+      <c r="A3" s="16"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1832,7 +2751,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -1849,7 +2768,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="14"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1864,7 +2783,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="16"/>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1877,7 +2796,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -1892,7 +2811,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
@@ -1905,7 +2824,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="3" t="s">
         <v>2</v>
       </c>
@@ -1918,7 +2837,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -1933,7 +2852,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
@@ -1946,7 +2865,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -1963,7 +2882,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="3" t="s">
         <v>20</v>
       </c>
@@ -1978,7 +2897,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1993,7 +2912,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -2007,10 +2926,10 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="13"/>
+      <c r="B20" s="20"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="13"/>
+      <c r="B21" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
update record screen soft url - Mirillis Action
</commit_message>
<xml_diff>
--- a/bill/record.xlsx
+++ b/bill/record.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alantop_dir\alantop_data\alantop_git\github\bill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAE9D83-6CE4-49AC-A8A3-74E314DAB54C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CFDAE8-5837-4C27-8202-3AEFFA5E77C2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="10.6 报名 Apply-10.7号打卡 " sheetId="7" r:id="rId1"/>
-    <sheet name="10.5 报名 Apply-10.6号打卡" sheetId="6" r:id="rId2"/>
-    <sheet name="10.4 报名 Apply " sheetId="5" r:id="rId3"/>
-    <sheet name="10.4 报名 Apply" sheetId="4" r:id="rId4"/>
-    <sheet name="10.3" sheetId="3" r:id="rId5"/>
-    <sheet name="10.2" sheetId="1" r:id="rId6"/>
+    <sheet name="10.8 报名 Apply-10.9号打卡" sheetId="9" r:id="rId1"/>
+    <sheet name="10.7 报名 Apply-10.8号打卡 " sheetId="8" r:id="rId2"/>
+    <sheet name="10.6 报名 Apply-10.7号打卡 " sheetId="7" r:id="rId3"/>
+    <sheet name="10.5 报名 Apply-10.6号打卡" sheetId="6" r:id="rId4"/>
+    <sheet name="10.4 报名 Apply " sheetId="5" r:id="rId5"/>
+    <sheet name="10.4 报名 Apply" sheetId="4" r:id="rId6"/>
+    <sheet name="10.3" sheetId="3" r:id="rId7"/>
+    <sheet name="10.2" sheetId="1" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="65">
   <si>
     <t>ju</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -269,6 +271,26 @@
   </si>
   <si>
     <t>10.5-10.11，10-7-10.13</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>芭芭农场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>银联云闪付</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中信居</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>悦动圈签到</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>绿色为报名</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -276,7 +298,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,6 +318,15 @@
       <color rgb="FFFF0000"/>
       <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -391,7 +422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -418,6 +449,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -712,19 +750,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9B029A4-88A2-46C8-B0E9-E61E955E93AB}">
-  <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81F8D7A-E99C-4A2C-B699-18239C685507}">
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>24</v>
@@ -751,8 +789,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -768,8 +806,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -783,8 +821,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -798,9 +836,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
-        <v>58</v>
-      </c>
+      <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
         <v>57</v>
       </c>
@@ -808,31 +844,25 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="3">
-        <v>1</v>
-      </c>
-      <c r="E5" s="14">
-        <v>1</v>
-      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="14"/>
       <c r="F5" s="3"/>
-      <c r="G5" s="3" t="s">
-        <v>32</v>
-      </c>
+      <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -846,23 +876,31 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="C7" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="14">
+        <v>1</v>
+      </c>
       <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -878,8 +916,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="21"/>
       <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
@@ -893,8 +931,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="18"/>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="21"/>
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
@@ -902,10 +940,12 @@
       <c r="D10" s="3">
         <v>1</v>
       </c>
-      <c r="E10" s="14">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3"/>
+      <c r="E10" s="18">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
       <c r="G10" s="3" t="s">
         <v>29</v>
       </c>
@@ -914,8 +954,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="22"/>
       <c r="B11" s="3" t="s">
         <v>52</v>
       </c>
@@ -929,8 +969,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -946,8 +986,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
       <c r="B13" s="3" t="s">
         <v>10</v>
       </c>
@@ -961,8 +1001,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -978,8 +1018,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="21"/>
       <c r="B15" s="3" t="s">
         <v>41</v>
       </c>
@@ -993,9 +1033,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="3"/>
-      <c r="G15" s="3" t="s">
-        <v>58</v>
-      </c>
+      <c r="G15" s="3"/>
       <c r="H15" s="3" t="s">
         <v>59</v>
       </c>
@@ -1003,8 +1041,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="21"/>
       <c r="B16" s="3" t="s">
         <v>39</v>
       </c>
@@ -1018,9 +1056,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="3"/>
-      <c r="G16" s="3" t="s">
-        <v>58</v>
-      </c>
+      <c r="G16" s="3"/>
       <c r="H16" s="3" t="s">
         <v>57</v>
       </c>
@@ -1028,8 +1064,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="22"/>
       <c r="B17" s="3" t="s">
         <v>47</v>
       </c>
@@ -1039,7 +1075,7 @@
       <c r="D17" s="3">
         <v>0</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="14">
         <v>1</v>
       </c>
       <c r="F17" s="3"/>
@@ -1051,8 +1087,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1068,8 +1104,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="19"/>
       <c r="B19" s="3" t="s">
         <v>12</v>
       </c>
@@ -1083,27 +1119,39 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1121,19 +1169,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1C76AF-BB5D-4CD7-A338-58E8ADB40F19}">
-  <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E58187-A6B7-4BD6-9A24-D6EDCBD2C48E}">
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>24</v>
@@ -1160,8 +1208,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1177,8 +1225,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -1192,8 +1240,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -1201,47 +1249,41 @@
         <v>4000</v>
       </c>
       <c r="D4" s="3">
-        <v>900</v>
-      </c>
-      <c r="E4" s="3">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>300</v>
+      </c>
+      <c r="E4" s="14">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0.5</v>
+      </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="I4" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="3">
-        <v>1</v>
-      </c>
-      <c r="E5" s="14">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>32</v>
-      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1255,8 +1297,441 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="14">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="21"/>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="21"/>
+      <c r="B10" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="14">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="22"/>
+      <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="21"/>
+      <c r="B15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="3">
+        <v>6666</v>
+      </c>
+      <c r="D15" s="3">
+        <v>300</v>
+      </c>
+      <c r="E15" s="14">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="21"/>
+      <c r="B16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D16" s="3">
+        <v>300</v>
+      </c>
+      <c r="E16" s="14">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="22"/>
+      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="14">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="19"/>
+      <c r="B19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A17"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9B029A4-88A2-46C8-B0E9-E61E955E93AB}">
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
+      <c r="B3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
+      <c r="B4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D4" s="3">
+        <v>300</v>
+      </c>
+      <c r="E4" s="14">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="14">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
+      <c r="B6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1270,8 +1745,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1287,8 +1762,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="21"/>
       <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
@@ -1302,8 +1777,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="18"/>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="21"/>
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1325,8 +1800,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="22"/>
       <c r="B11" s="3" t="s">
         <v>52</v>
       </c>
@@ -1340,8 +1815,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -1357,8 +1832,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
       <c r="B13" s="3" t="s">
         <v>10</v>
       </c>
@@ -1372,8 +1847,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1389,8 +1864,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="21"/>
       <c r="B15" s="3" t="s">
         <v>41</v>
       </c>
@@ -1400,22 +1875,24 @@
       <c r="D15" s="3">
         <v>300</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="14">
         <v>1</v>
       </c>
       <c r="F15" s="3">
-        <v>1</v>
-      </c>
-      <c r="G15" s="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H15" s="3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="I15" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="21"/>
       <c r="B16" s="3" t="s">
         <v>39</v>
       </c>
@@ -1423,24 +1900,26 @@
         <v>4000</v>
       </c>
       <c r="D16" s="3">
-        <v>900</v>
-      </c>
-      <c r="E16" s="3">
+        <v>300</v>
+      </c>
+      <c r="E16" s="14">
         <v>1</v>
       </c>
       <c r="F16" s="3">
-        <v>1</v>
-      </c>
-      <c r="G16" s="3"/>
+        <v>0.3</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H16" s="3" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="I16" s="3">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="22"/>
       <c r="B17" s="3" t="s">
         <v>47</v>
       </c>
@@ -1454,18 +1933,18 @@
         <v>1</v>
       </c>
       <c r="F17" s="3">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="I17" s="3">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1481,8 +1960,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="19"/>
       <c r="B19" s="3" t="s">
         <v>12</v>
       </c>
@@ -1496,22 +1975,447 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="2"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A17"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1C76AF-BB5D-4CD7-A338-58E8ADB40F19}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
+      <c r="B3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
+      <c r="B4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D4" s="3">
+        <v>900</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="14">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
+      <c r="B6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="21"/>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="21"/>
+      <c r="B10" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="14">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="22"/>
+      <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="21"/>
+      <c r="B15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="3">
+        <v>6666</v>
+      </c>
+      <c r="D15" s="3">
+        <v>300</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="21"/>
+      <c r="B16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D16" s="3">
+        <v>900</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="22"/>
+      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1</v>
+      </c>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="19"/>
+      <c r="B19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
     </row>
@@ -1530,20 +2434,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC38130-5053-47EB-A0EE-B1F3AFE32D40}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>24</v>
@@ -1576,8 +2480,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1595,8 +2499,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -1612,8 +2516,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -1641,8 +2545,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -1668,8 +2572,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1685,8 +2589,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1702,8 +2606,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1721,8 +2625,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="19"/>
       <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
@@ -1738,8 +2642,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="19"/>
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1763,8 +2667,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1782,8 +2686,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="19"/>
       <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
@@ -1799,8 +2703,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1820,8 +2724,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="19"/>
       <c r="B14" s="3" t="s">
         <v>41</v>
       </c>
@@ -1847,8 +2751,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="19"/>
       <c r="B15" s="3" t="s">
         <v>39</v>
       </c>
@@ -1876,8 +2780,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1895,8 +2799,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="19"/>
       <c r="B17" s="3" t="s">
         <v>12</v>
       </c>
@@ -1912,13 +2816,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="20"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="12"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="20"/>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B23" s="23"/>
       <c r="C23" s="12"/>
     </row>
   </sheetData>
@@ -1937,20 +2841,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9A0F91A-D02D-457B-B3D9-48656CF541FC}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>24</v>
@@ -1983,8 +2887,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2002,8 +2906,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -2019,8 +2923,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -2048,8 +2952,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -2075,8 +2979,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -2092,8 +2996,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
@@ -2109,8 +3013,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -2128,8 +3032,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="19"/>
       <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
@@ -2145,8 +3049,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="19"/>
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
@@ -2170,8 +3074,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -2189,8 +3093,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="19"/>
       <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
@@ -2206,8 +3110,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -2227,8 +3131,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="19"/>
       <c r="B14" s="3" t="s">
         <v>45</v>
       </c>
@@ -2254,8 +3158,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="19"/>
       <c r="B15" s="3" t="s">
         <v>46</v>
       </c>
@@ -2283,8 +3187,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -2302,8 +3206,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="19"/>
       <c r="B17" s="3" t="s">
         <v>12</v>
       </c>
@@ -2319,19 +3223,19 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="E18">
         <f>SUM(E2:E17)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="20"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="9"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="20"/>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B23" s="23"/>
       <c r="C23" s="9"/>
     </row>
   </sheetData>
@@ -2350,19 +3254,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42BB32C-5522-47CB-89EC-BA29E49614E8}">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
-    <col min="5" max="5" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>24</v>
@@ -2389,8 +3293,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2407,8 +3311,8 @@
         <v>0.3034722222222222</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -2420,8 +3324,8 @@
       </c>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="19" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -2441,8 +3345,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="19"/>
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -2462,8 +3366,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -2483,8 +3387,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -2506,8 +3410,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="19"/>
       <c r="B8" s="3" t="s">
         <v>28</v>
       </c>
@@ -2527,8 +3431,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="19"/>
       <c r="B9" s="3" t="s">
         <v>2</v>
       </c>
@@ -2546,8 +3450,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -2569,8 +3473,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="19"/>
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
@@ -2582,8 +3486,8 @@
       </c>
       <c r="G11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -2605,8 +3509,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
       <c r="B13" s="3" t="s">
         <v>20</v>
       </c>
@@ -2620,8 +3524,8 @@
       </c>
       <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -2643,8 +3547,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="19"/>
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -2656,7 +3560,7 @@
       </c>
       <c r="G15" s="6"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2664,13 +3568,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="20"/>
+      <c r="B20" s="23"/>
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="20"/>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="23"/>
       <c r="C21" s="1"/>
     </row>
   </sheetData>
@@ -2689,18 +3593,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -2718,8 +3622,8 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2735,8 +3639,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -2750,8 +3654,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="19" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -2767,8 +3671,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="19"/>
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -2782,8 +3686,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -2795,8 +3699,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -2810,8 +3714,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="19"/>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
@@ -2823,8 +3727,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="19"/>
       <c r="B9" s="3" t="s">
         <v>2</v>
       </c>
@@ -2836,8 +3740,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -2851,8 +3755,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="19"/>
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
@@ -2864,8 +3768,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -2881,8 +3785,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
       <c r="B13" s="3" t="s">
         <v>20</v>
       </c>
@@ -2896,8 +3800,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -2911,8 +3815,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="19"/>
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -2924,12 +3828,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="20"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="20"/>
+      <c r="B20" s="23"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B21" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>